<commit_message>
Fix generic filler descriptions in Units 3-4 coding questions
Same bug as Unit 2: 10 of 40 questions per unit had placeholder
descriptions that never stated the actual rule/formula. Rewrote each
with a real scenario and explicit logic, verified against existing
solutions/test cases. Unit 4's fixes include two pattern-printing
questions (Number Triangle, Grid Border Stars) that exercise nested
loops, per the meeting's ask for more pattern-based coding questions.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/Question Bank/Coding Questions/Unit 3 - Control Flow/Unit 3 - Control Flow - Coding Questions.xlsx
+++ b/content/Question Bank/Coding Questions/Unit 3 - Control Flow/Unit 3 - Control Flow - Coding Questions.xlsx
@@ -1913,7 +1913,8 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A community lucky-draw booth uses locker token numbers to decide who gets to enter the bonus round - only even-numbered tokens qualify. Write a program that reads a token number and prints whether it is eligible. Print `Eligible` if the number is even, and `Not Eligible` if it is odd.
+          <t>A lucky-draw counter at a college fest only lets in visitors whose token number is even, since odd tokens go to a different queue.
+Write a program that reads a visitor's token number and prints `Eligible` if the number is even, and `Not Eligible` otherwise.
 ### Input Format
 - Line 1: Token number
 ### Output Format
@@ -1921,9 +1922,9 @@
 Eligible
 ```
 ### Example Walkthrough
-In the sample, the token number is `2`. Since `2 % 2 == 0`, the number is even, so the program prints `Eligible`. A token number of `3` would instead print `Not Eligible`.
+In the sample, the token is 2. Since 2 is divisible by 2 with no remainder, it is even, so the program prints `Eligible`. A token of 3 would instead print `Not Eligible`.
 ### Constraints
-- All numeric inputs are valid integers in the ranges implied by the examples.
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -2069,7 +2070,8 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A skills-certification platform scores every attempt and needs to instantly label it before generating the certificate. Any score of 40 or above counts as a passing attempt. Write a program that reads an attempt's score and prints exactly `Pass` if the score is 40 or more, and exactly `Fail` otherwise.
+          <t>A results portal needs to instantly label each student's score as a pass or a fail the moment it is entered, before the full report card is generated. The passing cutoff is a score of 40 or more.
+Write a program that reads a student's score and prints `Pass` if the score is 40 or more, and `Fail` otherwise.
 ### Input Format
 - Line 1: Score
 ### Output Format
@@ -2077,9 +2079,9 @@
 Pass
 ```
 ### Example Walkthrough
-In the sample, the score is `40`. Since `40 &gt;= 40`, the passing condition is true, so the program prints `Pass`. A score of `39` would instead print `Fail`.
+In the sample, the score is 40. Since 40 is greater than or equal to 40, the program prints `Pass`. A score of 39 would instead print `Fail`.
 ### Constraints
-- All numeric inputs are valid numbers in the ranges implied by the examples.
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -3719,7 +3721,8 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A weather-monitoring app sends out a heat alert whenever the recorded temperature crosses a safe threshold. Write a program that reads a temperature reading (in Celsius) and prints whether it should trigger a heat alert. Print `Hot` if the temperature is strictly greater than 35, and `Normal` otherwise.
+          <t>A weather station's alert board flashes a warning whenever the recorded temperature crosses into dangerously hot territory, defined as anything above 35 degrees.
+Write a program that reads the current temperature as a decimal number and prints `Hot` if it is strictly greater than 35, and `Normal` otherwise.
 ### Input Format
 - Line 1: Temperature
 ### Output Format
@@ -3727,7 +3730,7 @@
 Hot
 ```
 ### Example Walkthrough
-In the sample, the temperature is `36`. Since `36 &gt; 35`, the program prints `Hot`. A temperature of `35` would instead print `Normal`, since it does not exceed the threshold.
+In the sample, the temperature is 36. Since 36 is greater than 35, the program prints `Hot`. A temperature of exactly 35 would instead print `Normal`.
 ### Constraints
 - All numeric inputs are valid numbers in the ranges implied by the examples.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
@@ -3875,18 +3878,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A quick scoreboard widget compares two submitted values and highlights the larger one. Write a program that reads two numbers and prints the larger of the two. If the two numbers are equal, print that common value.
+          <t>A scoreboard app compares two contestants' scores after every round and highlights whichever one is ahead, breaking ties in favor of the first contestant.
+Write a program that reads two scores and prints the larger of the two; if they are equal, print the first score.
 ### Input Format
-- Line 1: First number
-- Line 2: Second number
+- Line 1: First score
+- Line 2: Second score
 ### Output Format
 ```
 5
 ```
 ### Example Walkthrough
-In the sample, the first number is `5` and the second is `3`. Since `5` is greater than `3`, the program prints `5`.
+In the sample, the first score is 5 and the second is 3. Since 5 is greater than or equal to 3, the program prints `5`.
 ### Constraints
-- All numeric inputs are valid integers in the ranges implied by the examples.
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -5437,7 +5441,8 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>An online course dashboard sorts learners into performance bands based on their quiz score, so instructors know who needs extra help. Write a program that reads a score and prints the grade band: `A` for scores of 90 or above, `B` for scores from 75 up to (but not including) 90, `C` for scores from 50 up to (but not including) 75, and `Needs Practice` for anything below 50.
+          <t>A results portal converts every numeric score into a letter grade band before displaying it on the student dashboard. The bands are: 90 or above is `A`, 75 up to 89 is `B`, 50 up to 74 is `C`, and anything below 50 is `Needs Practice`.
+Write a program that reads a student's score and prints the correct grade band using these cutoffs.
 ### Input Format
 - Line 1: Score
 ### Output Format
@@ -5445,9 +5450,9 @@
 A
 ```
 ### Example Walkthrough
-In the sample, the score is `95`. Since `95` is 90 or above, the program prints `A`.
+In the sample, the score is 95. Since 95 is 90 or above, the program prints `A`. A score of 80 would print `B`, 65 would print `C`, and 40 would print `Needs Practice`.
 ### Constraints
-- All numeric inputs are valid numbers in the ranges implied by the examples.
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -5596,18 +5601,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A campus portal grants different levels of access depending on a user's role and whether their account is currently active. Write a program that reads a role and an account status (`active` or `inactive`), then prints the access level. If the account is inactive, print `No Access` regardless of role. If the account is active: print `Full Access` for role `admin`, `Learning Access` for role `student`, and `Limited Access` for any other role.
+          <t>A campus portal decides what a logged-in user can see based on two things: their account status and their role. If the account is not `active`, the user gets no access regardless of role. If it is active, an `admin` gets full access, a `student` gets learning access, and anyone else gets limited access.
+Write a program that reads the role and the status, then prints exactly one of `Full Access`, `Learning Access`, `Limited Access`, or `No Access` following this rule.
 ### Input Format
 - Line 1: Role
-- Line 2: Account status (`active` or `inactive`)
+- Line 2: Status (`active` or any other value)
 ### Output Format
 ```
 Full Access
 ```
 ### Example Walkthrough
-In the sample, the role is `admin` and the status is `active`. Since the account is active and the role is `admin`, the program prints `Full Access`.
+In the sample, the role is admin and the status is active. Since the status is active and the role is admin, the program prints `Full Access`.
 ### Constraints
-- All inputs follow the exact casing and format shown in the examples.
+- Role and status are valid strings with no leading or trailing spaces.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -5765,7 +5771,8 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A scheduling system tags each day code coming from an upstream system as a weekday or weekend slot before assigning shifts. Write a program that reads a three-letter day code and prints its type. Print `Weekend` for `SAT` or `SUN`, `Weekday` for `MON`, `TUE`, `WED`, `THU`, or `FRI`, and `Unknown` for any other code (the check is case-sensitive, so a lowercase code like `sat` also counts as `Unknown`).
+          <t>A hostel mess planning tool reads a three-letter day code and needs to know whether it falls on a weekday or a weekend, so it can plan the right menu. `SAT` and `SUN` are weekends, `MON` through `FRI` are weekdays, and anything else is not a recognized code.
+Write a program that reads a three-letter day code and prints `Weekend`, `Weekday`, or `Unknown` accordingly. The check is case-sensitive.
 ### Input Format
 - Line 1: Day code
 ### Output Format
@@ -5773,9 +5780,9 @@
 Weekday
 ```
 ### Example Walkthrough
-In the sample, the day code is `MON`. Since `MON` is one of the weekday codes, the program prints `Weekday`.
+In the sample, the code is MON. Since MON is one of the weekday codes, the program prints `Weekday`. A code of SAT would print `Weekend`, and a lowercase code like sat would print `Unknown` since the check is case-sensitive.
 ### Constraints
-- Day codes are provided in uppercase unless intentionally testing the Unknown case.
+- Day code is a valid string with no leading or trailing spaces.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -7301,18 +7308,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A university scholarship committee screens applicants using both their marks and attendance before deciding who qualifies outright, who goes on a waitlist, and who is turned down. Write a program that reads a student's marks and attendance percentage, then prints the decision. Print `Eligible` if marks are 85 or above AND attendance is 90 or above; print `Waitlist` if only one of those two conditions is met; print `Not Eligible` if neither condition is met.
+          <t>A scholarship committee reviews each applicant's marks percentage and attendance percentage together. An applicant is fully `Eligible` only when both marks are at least 85 and attendance is at least 90; if only one of the two conditions is met they go on a `Waitlist`; if neither is met they are `Not Eligible`.
+Write a program that reads the marks percentage and the attendance percentage, then prints `Eligible`, `Waitlist`, or `Not Eligible` following this rule.
 ### Input Format
-- Line 1: Marks
+- Line 1: Marks percentage
 - Line 2: Attendance percentage
 ### Output Format
 ```
 Eligible
 ```
 ### Example Walkthrough
-In the sample, the marks are `90` and the attendance is `95`. Since both marks (`&gt;= 85`) and attendance (`&gt;= 90`) meet the thresholds, the program prints `Eligible`.
+In the sample, marks are 90 and attendance is 95. Since marks are at least 85 and attendance is at least 90, both conditions are met, so the program prints `Eligible`. Marks of 85 with attendance of 89 would meet only one condition and print `Waitlist`.
 ### Constraints
-- All numeric inputs are valid numbers in the ranges implied by the examples.
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -7468,7 +7476,8 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A geometry teaching tool checks three submitted side lengths and classifies the resulting shape, but first it must confirm the sides can actually form a triangle. Write a program that reads three side lengths a, b, and c, then prints the triangle type. Print `Invalid` if any side is zero or negative, or if the triangle inequality fails (the sum of any two sides is not strictly greater than the third). Otherwise, print `Equilateral` if all three sides are equal, `Isosceles` if exactly two sides are equal, and `Scalene` if all three sides are different.
+          <t>A geometry teaching app checks three side lengths entered by a student and classifies the shape before drawing it. The sides must each be positive and satisfy the triangle inequality (no side can be greater than or equal to the sum of the other two), otherwise the shape is `Invalid`. A valid triangle with all three sides equal is `Equilateral`, one with exactly two equal sides is `Isosceles`, and one with all different sides is `Scalene`.
+Write a program that reads three side lengths and prints `Invalid`, `Equilateral`, `Isosceles`, or `Scalene` following this rule.
 ### Input Format
 - Line 1: Side a
 - Line 2: Side b
@@ -7478,9 +7487,9 @@
 Equilateral
 ```
 ### Example Walkthrough
-In the sample, the sides are `3`, `3`, and `3`. They satisfy the triangle inequality, and all three sides are equal, so the program prints `Equilateral`.
+In the sample, the sides are 3, 3, and 3. They form a valid triangle and all three sides are equal, so the program prints `Equilateral`. Sides 3, 3, 4 would print `Isosceles`, and sides 1, 2, 3 would print `Invalid` since 1 + 2 is not greater than 3.
 ### Constraints
-- All numeric inputs are valid integers in the ranges implied by the examples.
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -7643,16 +7652,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A calculator utility divides two numbers submitted by a user, but must guard against a divide-by-zero crash. Write a program that reads a numerator and a divisor, then prints the result. If the divisor is 0, print `Cannot divide`; otherwise print the numerator divided by the divisor as a floating-point value.
+          <t>A calculator widget divides two numbers a user enters, but must guard against a zero denominator instead of letting the app crash.
+Write a program that reads two decimal numbers and prints their quotient (first divided by second); if the second number is 0, print `Cannot divide` instead.
 ### Input Format
-- Line 1: Numerator
-- Line 2: Divisor
+- Line 1: First number
+- Line 2: Second number
 ### Output Format
 ```
 5.0
 ```
 ### Example Walkthrough
-In the sample, the numerator is `10` and the divisor is `2`. Since the divisor is not `0`, the program prints `10 / 2`, which is `5.0`.
+In the sample, the numbers are 10 and 2. Since 2 is not 0, the program divides 10 by 2 and prints `5.0`. If the second number were 0, it would print `Cannot divide` instead.
 ### Constraints
 - All numeric inputs are valid numbers in the ranges implied by the examples.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>

</xml_diff>